<commit_message>
estudo: lendo e alterando a planilha
</commit_message>
<xml_diff>
--- a/modulos_com_python/aula337_openpyxl/workbook.xlsx
+++ b/modulos_com_python/aula337_openpyxl/workbook.xlsx
@@ -453,7 +453,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C3" t="n">
         <v>9.699999999999999</v>
@@ -479,7 +479,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C5" t="n">
         <v>10</v>

</xml_diff>